<commit_message>
Adiciona requeijão e atualiza iogurte natural na planilha
- Requeijão (Laticínios, Moderar — rico em gordura saturada/sódio)
- Iogurte natural renomeado para deixar explícito 'sem açúcar'

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1368,7 +1368,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Iogurte natural desnatado</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -1388,192 +1388,192 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Sem açúcar adicionado</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>1 colher de sopa (≈15 g)</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>à vontade</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
+          <t>Suco natural sem açúcar</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="11" t="inlineStr">
+        <is>
           <t>Bebida alcoólica</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>evitar</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>Evitar</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Piora diretamente os triglicerídeos</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Doces e Sobremesas</t>
         </is>
       </c>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="10" t="n"/>
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="10" t="n"/>
-      <c r="F31" s="10" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Açúcar refinado</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1591,188 +1591,215 @@
           <t>Evitar</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr"/>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="11" t="inlineStr">
         <is>
+          <t>Doces industrializados</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
           <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>10 g</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="F34" s="11" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Gorduras e Temperos</t>
         </is>
       </c>
-      <c r="B35" s="10" t="n"/>
-      <c r="C35" s="10" t="n"/>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="10" t="n"/>
-      <c r="F35" s="10" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>Azeite de oliva extra virgem</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>1-2 colheres de sopa</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F36" s="11" t="inlineStr"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E37" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
+          <t>Preferir azeite</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="11" t="inlineStr">
         <is>
+          <t>Sal</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>&lt; 5 g no total</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Somar sal de cozinha + industrializados</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
           <t>Ervas e temperos naturais</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="D39" s="12" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F39" s="11" t="inlineStr"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="10" t="n"/>
-      <c r="E40" s="10" t="n"/>
-      <c r="F40" s="10" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="10" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="D41" s="12" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F41" s="11" t="inlineStr">
+      <c r="F42" s="11" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="16" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Lista com os alimentos acrescentados até agora — não é uma lista completa. Use a skill 'adicionar-alimento' (ex.: "adicione sucrilhos") para ir acrescentando novos itens aos poucos.</t>
         </is>
@@ -1780,16 +1807,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lista de medicações da alta e interações com alimentos
- referencia/dados-consulta-e-alimentacao.md: nova seção 1a com as 5
  medicações da receita de 03/09/2026 (dose, posologia, indicação) e as
  interações com alimentos já identificadas; checklist de pendências
  atualizado
- referencia/historico-tratamento.md: linha do tempo e seção nova sobre
  a receita de alta
- planilha: aba 'Cuidados na Alimentação' com a lista de medicações e
  4 avisos de interação medicamentosa (Ticagrelor x toranja, Enalapril
  x potássio/sal light, Aspirina+Ticagrelor x álcool, Rosucor x arroz
  de levedura vermelha); aba 'Alimentos e Quantidades' com toranja,
  suco de toranja e sal light marcados como Evitar
- skill adicionar-alimento: instruída a sempre checar essas interações
  ao classificar um alimento novo

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -703,22 +703,70 @@
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Aviso pendente — medicação</t>
+          <t>Medicações em uso (receita 03/09/2026)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Lista de medicações da alta ainda não preenchida. Existem interações conhecidas entre alimentos e medicações comuns pós-IAM (ex.: anticoagulantes como varfarina e vegetais verde-escuros ricos em vitamina K). Revisar esta planilha assim que a lista de medicações estiver disponível.</t>
+          <t>Aspirina Prevent 100mg (1x/dia, almoço) e Ticagrelor 90mg (12/12h, por 1 ano) — antiagregantes plaquetários; Rosucor (rosuvastatina) 20mg, 2 comprimidos 1x/dia, e Ezetimiba 10mg 1x/dia — colesterol; Maleato de Enalapril 5mg 12/12h — coração/pressão (médico alertou para cuidado com pressão baixa). Todas de uso contínuo — não interromper sem falar com o cardiologista, em especial a dupla Aspirina + Ticagrelor (risco de trombose no stent).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Interação medicamentosa — Ticagrelor</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Toranja/grapefruit (fruta ou suco) aumenta o nível de Ticagrelor no sangue e o risco de sangramento — evitar completamente enquanto estiver em uso do medicamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Interação medicamentosa — Enalapril</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Enalapril pode elevar o potássio do sangue. Evitar sal light/substitutos de sal (ricos em cloreto de potássio) e suplementos de potássio sem orientação médica — atenção redobrada enquanto a função renal ainda está em investigação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Interação medicamentosa — Aspirina + Ticagrelor</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>A dupla antiagregação (esquema padrão por 1 ano pós-stent) já aumenta o risco de sangramento; álcool amplifica esse risco — reforça a orientação de evitar bebida alcoólica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Interação medicamentosa — Rosucor (estatina)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Evitar suplementos de 'arroz de levedura vermelha' (red yeast rice), que agem como uma estatina natural e podem somar toxicidade com a Rosucor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Leitura de rótulos</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Ao comprar um produto industrializado, olhar sempre: sódio por porção, açúcares totais/adicionados, e a lista de ingredientes procurando 'gordura hidrogenada' ou 'gordura trans'. Prefira produtos com menos ingredientes e sem açúcar adicionado.</t>
         </is>
@@ -850,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1056,45 +1104,49 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Toranja / grapefruit</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Interage com o Ticagrelor (aumenta o nível do remédio no sangue e o risco de sangramento) — evitar completamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Grãos e Cereais</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Arroz integral</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>200 g (cozido)</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>quase todo dia</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Arroz branco</t>
+          <t>Arroz integral</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
@@ -1104,113 +1156,109 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Preferir integral no restante da semana</t>
-        </is>
-      </c>
+          <t>quase todo dia</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Aveia</t>
+          <t>Arroz branco</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>2 colheres de sopa</t>
+          <t>200 g (cozido)</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Ajuda a reduzir colesterol</t>
+          <t>Preferir integral no restante da semana</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="11" t="inlineStr">
         <is>
+          <t>Aveia</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>2 colheres de sopa</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Ajuda a reduzir colesterol</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
           <t>Pão integral</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>2 fatias</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>1x/dia</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Proteínas</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Peixe</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>150 g</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Fonte de ômega-3</t>
-        </is>
-      </c>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Frango sem pele</t>
+          <t>Peixe</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -1220,7 +1268,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>quase todo dia</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -1228,12 +1276,16 @@
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Fonte de ômega-3</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Carne vermelha magra</t>
+          <t>Frango sem pele</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -1243,337 +1295,348 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>1x/semana</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Preferir cortes magros</t>
-        </is>
-      </c>
+          <t>quase todo dia</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Ovo</t>
+          <t>Carne vermelha magra</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>150 g</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>até 5x/semana</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr"/>
+          <t>1x/semana</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Preferir cortes magros</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="11" t="inlineStr">
         <is>
+          <t>Ovo</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>1 unidade</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>até 5x/semana</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
           <t>Feijão / leguminosas</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>1 concha</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>1x/dia</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Laticínios</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Leite desnatado</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>200 ml</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Queijo branco</t>
+          <t>Leite desnatado</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>30 g</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Atenção ao sódio</t>
-        </is>
-      </c>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Queijo branco</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Prefira sempre a versão sem açúcar adicionado</t>
+          <t>Atenção ao sódio</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="11" t="inlineStr">
         <is>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>1 unidade</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
           <t>Requeijão</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>1 colher de sopa (≈15 g)</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>à vontade</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Suco de toranja / grapefruit</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>evitar</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Evitar</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Piora diretamente os triglicerídeos</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Doces e Sobremesas</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="10" t="n"/>
-      <c r="F32" s="10" t="n"/>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Interage com o Ticagrelor (aumenta o nível do remédio no sangue e o risco de sangramento) — evitar completamente.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Bebida alcoólica</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1593,213 +1656,279 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>Doces industrializados</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="inlineStr"/>
+          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Doces e Sobremesas</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>10 g</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>Gorduras e Temperos</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="10" t="n"/>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Doces industrializados</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Azeite de oliva extra virgem</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>1-2 colheres de sopa</t>
+          <t>10 g</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="inlineStr"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Manteiga</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F38" s="11" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Gorduras e Temperos</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F39" s="11" t="inlineStr">
-        <is>
-          <t>Somar sal de cozinha + industrializados</t>
-        </is>
-      </c>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>Preferir azeite</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Sal</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>&lt; 5 g no total</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>Vegetais e Verduras</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="n"/>
-      <c r="C41" s="10" t="n"/>
-      <c r="D41" s="10" t="n"/>
-      <c r="E41" s="10" t="n"/>
-      <c r="F41" s="10" t="n"/>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>Somar sal de cozinha + industrializados</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="11" t="inlineStr">
         <is>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>à vontade</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Vegetais e Verduras</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="11" t="inlineStr">
+        <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="C42" s="12" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F42" s="11" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>Lista com os alimentos acrescentados até agora — não é uma lista completa. Use a skill 'adicionar-alimento' (ex.: "adicione sucrilhos") para ir acrescentando novos itens aos poucos.</t>
         </is>
@@ -1807,16 +1936,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A47:F47"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona mussarela à planilha
- Mussarela (Laticínios, Moderar) — 30g, 2x/semana, café da manhã/lanche
- Mais gordura saturada e sódio que o queijo branco já cadastrado

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -1061,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1606,266 +1606,266 @@
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Prefira sempre a versão sem açúcar adicionado</t>
+          <t>Mais gordura saturada e sódio que o queijo branco; prefira o queijo branco no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="11" t="inlineStr">
         <is>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>1 unidade</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="11" t="inlineStr">
+        <is>
           <t>Requeijão</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>1 colher de sopa (≈15 g)</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="10" t="n"/>
-      <c r="F27" s="10" t="n"/>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>à vontade</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
         <is>
+          <t>Suco de toranja / grapefruit</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
           <t>Bebida alcoólica</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>evitar</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>Evitar</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>Doces e Sobremesas</t>
         </is>
       </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>Açúcar refinado</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E35" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -1883,215 +1883,242 @@
           <t>Evitar</t>
         </is>
       </c>
-      <c r="F36" s="11" t="inlineStr"/>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="11" t="inlineStr">
         <is>
+          <t>Doces industrializados</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
           <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>10 g</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr">
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="F37" s="11" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
         <is>
           <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Gorduras e Temperos</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="10" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>Azeite de oliva extra virgem</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>1-2 colheres de sopa</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="F39" s="11" t="inlineStr"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="E41" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
+          <t>Preferir azeite</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+          <t>Somar sal de cozinha + industrializados</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="11" t="inlineStr">
         <is>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="11" t="inlineStr">
+        <is>
           <t>Ervas e temperos naturais</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E44" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F43" s="11" t="inlineStr"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="F44" s="11" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="B44" s="10" t="n"/>
-      <c r="C44" s="10" t="n"/>
-      <c r="D44" s="10" t="n"/>
-      <c r="E44" s="10" t="n"/>
-      <c r="F44" s="10" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="B45" s="11" t="inlineStr">
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="10" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="F45" s="11" t="inlineStr">
+      <c r="F46" s="11" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>Lista com os alimentos acrescentados até agora — não é uma lista completa. Use a skill 'adicionar-alimento' (ex.: "adicione sucrilhos") para ir acrescentando novos itens aos poucos.</t>
         </is>
@@ -2099,16 +2126,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A45:F45"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A39:F39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3795,7 +3822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:U36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4889,7 +4916,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -4963,7 +4990,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -5023,7 +5050,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -5033,7 +5060,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -5093,17 +5120,17 @@
       <c r="J17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
           <t>Suco natural sem açúcar</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -5167,12 +5194,12 @@
       <c r="J18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -5189,7 +5216,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5199,22 +5226,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1x/dia</t>
+          <t>2x/semana</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Prefira sempre a versão sem açúcar adicionado</t>
+          <t>Mais gordura saturada e sódio que o queijo branco; prefira o queijo branco no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5231,12 +5258,12 @@
       <c r="J19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -5253,7 +5280,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5263,22 +5290,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1 colher de sopa (≈15 g)</t>
+          <t>1 unidade</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2x/semana</t>
+          <t>1x/dia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5295,12 +5322,12 @@
       <c r="J20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -5317,58 +5344,54 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Laticínios</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>1 colher de sopa (≈15 g)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -5385,7 +5408,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5395,25 +5418,25 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>X</t>
@@ -5427,6 +5450,16 @@
       <c r="J22" t="inlineStr">
         <is>
           <t>X</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Manteiga</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -5443,7 +5476,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5453,32 +5486,40 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>Proteínas|Jantar</t>
@@ -5493,7 +5534,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5503,24 +5544,20 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>X</t>
@@ -5547,7 +5584,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5557,22 +5594,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5601,7 +5638,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5626,21 +5663,21 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
           <t>Gorduras e Temperos|Jantar</t>
@@ -5655,12 +5692,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Bebida alcoólica</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Doces e Sobremesas</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5680,24 +5717,16 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>X</t>
@@ -5717,7 +5746,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5740,20 +5769,36 @@
           <t>evitar</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5763,24 +5808,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10 g</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
@@ -5793,47 +5834,47 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Azeite de oliva extra virgem</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Gorduras e Temperos</t>
+          <t>Doces e Sobremesas</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1-2 colheres de sopa</t>
+          <t>10 g</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5843,37 +5884,37 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5883,41 +5924,37 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>todos os dias</t>
+          <t>evitar</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Preferir azeite</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5927,22 +5964,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>todos os dias</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+          <t>Somar sal de cozinha + industrializados</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -5961,7 +5998,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5971,20 +6008,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
@@ -6001,50 +6042,90 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gorduras e Temperos</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>à vontade</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>X</t>
         </is>

</xml_diff>

<commit_message>
Renomeia e ajusta pão integral e queijo branco na planilha
- 'Pão integral' -> 'Pão de forma integral' (mesmo alimento, nome mais
  específico pedido pelo usuário; porção/frequência/classificação
  mantidas)
- 'Queijo branco' -> 'Queijo branco frescal', com classificação subindo
  de Moderar para Liberado: o tipo frescal (ex. Minas frescal) é fresco,
  sem cura/salga pesada, com bem menos sódio e gordura que queijo curado
- Observação da Mussarela atualizada para referenciar o queijo frescal

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -983,7 +983,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>1/2 do prato: vegetais e salada (à vontade, tempero simples com azeite/limão). 1/4 do prato: proteína magra grelhada/assada (peixe, frango sem pele, ovo, leguminosas). 1/4 do prato: carboidrato integral (arroz integral, batata-doce, mandioca, pão integral) em porção moderada.</t>
+          <t>1/2 do prato: vegetais e salada (à vontade, tempero simples com azeite/limão). 1/4 do prato: proteína magra grelhada/assada (peixe, frango sem pele, ovo, leguminosas). 1/4 do prato: carboidrato integral (arroz integral, batata-doce, mandioca, pão de forma integral) em porção moderada.</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Pão integral</t>
+          <t>Pão de forma integral</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Queijo branco</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -1592,14 +1592,14 @@
           <t>3x/semana</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Atenção ao sódio</t>
+          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Mais gordura saturada e sódio que o queijo branco; prefira o queijo branco no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Pão integral</t>
+          <t>Pão de forma integral</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -4290,7 +4290,7 @@
       <c r="J6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Pão integral</t>
+          <t>Pão de forma integral</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -4618,7 +4618,7 @@
       <c r="J10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -4650,7 +4650,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pão integral</t>
+          <t>Pão de forma integral</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4688,7 +4688,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Queijo branco</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Queijo branco</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -5145,14 +5145,14 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Pão integral</t>
+          <t>Pão de forma integral</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Queijo branco</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Atenção ao sódio</t>
+          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mais gordura saturada e sódio que o queijo branco; prefira o queijo branco no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona pão francês integral (Mambo) à planilha
- Pão francês integral/multigrãos (Grãos e Cereais, Liberado) - marca
  Mambo, com dados reais do rótulo (120 kcal e 208 mg de sódio por
  porção de 50g, 1,6 g de fibras, sem açúcar adicionado)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -1061,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1447,53 +1447,57 @@
       <c r="G15" s="13" t="inlineStr"/>
       <c r="H15" s="12" t="inlineStr"/>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Pão francês integral (multigrãos)</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Mambo</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>1 unidade (~67 g)</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr"/>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Rótulo real (porção 50 g/meia unidade): 120 kcal, 208 mg de sódio, 1,6 g de fibras, sem açúcar adicionado. Com centeio, gergelim e linhaça — boa fonte de fibra, mas sódio moderado como a maioria dos pães; contém glúten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Proteínas</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="11" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Peixe</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="inlineStr"/>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>150 g</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr"/>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>Fonte de ômega-3</t>
-        </is>
-      </c>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Frango sem pele</t>
+          <t>Peixe</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr"/>
@@ -1504,7 +1508,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>quase todo dia</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -1513,12 +1517,16 @@
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="12" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Fonte de ômega-3</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Carne vermelha magra</t>
+          <t>Frango sem pele</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr"/>
@@ -1529,61 +1537,61 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>1x/semana</t>
-        </is>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>quase todo dia</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr"/>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>Preferir cortes magros</t>
-        </is>
-      </c>
+      <c r="H19" s="12" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>Ovo</t>
+          <t>Carne vermelha magra</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr"/>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>150 g</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>até 5x/semana</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>1x/semana</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr"/>
-      <c r="H20" s="12" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Preferir cortes magros</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Feijão / leguminosas</t>
+          <t>Ovo</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr"/>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>1 concha</t>
+          <t>1 unidade</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>1x/dia</t>
+          <t>até 5x/semana</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
@@ -1594,60 +1602,60 @@
       <c r="G21" s="13" t="inlineStr"/>
       <c r="H21" s="12" t="inlineStr"/>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Feijão / leguminosas</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr"/>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>1 concha</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Laticínios</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
-      <c r="H22" s="11" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Leite desnatado</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr"/>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>200 ml</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr"/>
-      <c r="H23" s="12" t="inlineStr"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="11" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Queijo branco frescal</t>
+          <t>Leite desnatado</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr"/>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>30 g</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>3x/semana</t>
+          <t>1x/dia</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -1656,26 +1664,18 @@
         </is>
       </c>
       <c r="G24" s="13" t="inlineStr"/>
-      <c r="H24" s="12" t="inlineStr">
-        <is>
-          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
-        </is>
-      </c>
+      <c r="H24" s="12" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Queijo frescal light</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>Polenghi</t>
-        </is>
-      </c>
+          <t>Queijo branco frescal</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr"/>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>30 g (1 fatia)</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -1691,252 +1691,256 @@
       <c r="G25" s="13" t="inlineStr"/>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>Rótulo real: 41 kcal e 105 mg de sódio por porção (bem abaixo de queijos comuns), 1,5 g de gordura saturada, sem açúcar adicionado. Contém lactose; sem glúten; pode conter soja.</t>
+          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Mussarela</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr"/>
+          <t>Queijo frescal light</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Polenghi</t>
+        </is>
+      </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>30 g</t>
+          <t>30 g (1 fatia)</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr"/>
       <c r="H26" s="12" t="inlineStr">
         <is>
-          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Rótulo real: 41 kcal e 105 mg de sódio por porção (bem abaixo de queijos comuns), 1,5 g de gordura saturada, sem açúcar adicionado. Contém lactose; sem glúten; pode conter soja.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr"/>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G27" s="13" t="inlineStr"/>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>Prefira sempre a versão sem açúcar adicionado</t>
+          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr"/>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>1 colher de sopa (≈15 g)</t>
+          <t>1 unidade</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F28" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr"/>
       <c r="H28" s="12" t="inlineStr">
         <is>
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr"/>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>1 colher de sopa (≈15 g)</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
           <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="11" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr"/>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>à vontade</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr"/>
-      <c r="H30" s="12" t="inlineStr"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="11" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr"/>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F31" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G31" s="13" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+      <c r="H31" s="12" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr"/>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr"/>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr"/>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G33" s="13" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+      <c r="H33" s="12" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr"/>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F34" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr"/>
       <c r="H34" s="12" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr"/>
@@ -1958,57 +1962,57 @@
       <c r="G35" s="13" t="inlineStr"/>
       <c r="H35" s="12" t="inlineStr">
         <is>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Bebida alcoólica</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr"/>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr"/>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
           <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Doces e Sobremesas</t>
         </is>
       </c>
-      <c r="B36" s="11" t="n"/>
-      <c r="C36" s="11" t="n"/>
-      <c r="D36" s="11" t="n"/>
-      <c r="E36" s="11" t="n"/>
-      <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="n"/>
-      <c r="H36" s="11" t="n"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>Açúcar refinado</t>
-        </is>
-      </c>
-      <c r="C37" s="13" t="inlineStr"/>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F37" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="G37" s="13" t="inlineStr"/>
-      <c r="H37" s="12" t="inlineStr">
-        <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="11" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr"/>
@@ -2028,233 +2032,262 @@
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr"/>
-      <c r="H38" s="12" t="inlineStr"/>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr"/>
       <c r="D39" s="13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr"/>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Chocolate amargo (70%+)</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr"/>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
           <t>10 g</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="F39" s="15" t="inlineStr">
+      <c r="F40" s="15" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="G39" s="13" t="inlineStr"/>
-      <c r="H39" s="12" t="inlineStr">
+      <c r="G40" s="13" t="inlineStr"/>
+      <c r="H40" s="12" t="inlineStr">
         <is>
           <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Gorduras e Temperos</t>
         </is>
       </c>
-      <c r="B40" s="11" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="11" t="n"/>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="11" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>Azeite de oliva extra virgem</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr"/>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>1-2 colheres de sopa</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F41" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G41" s="13" t="inlineStr"/>
-      <c r="H41" s="12" t="inlineStr"/>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr"/>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F42" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G42" s="13" t="inlineStr"/>
-      <c r="H42" s="12" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
+      <c r="H42" s="12" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr"/>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F43" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="G43" s="13" t="inlineStr"/>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
+          <t>Preferir azeite</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr"/>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F44" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G44" s="13" t="inlineStr"/>
       <c r="H44" s="12" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+          <t>Somar sal de cozinha + industrializados</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr"/>
       <c r="D45" s="13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G45" s="13" t="inlineStr"/>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr"/>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F45" s="14" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="G45" s="13" t="inlineStr"/>
-      <c r="H45" s="12" t="inlineStr"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="10" t="inlineStr">
+      <c r="G46" s="13" t="inlineStr"/>
+      <c r="H46" s="12" t="inlineStr"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="B46" s="11" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="11" t="n"/>
-      <c r="E46" s="11" t="n"/>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="11" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="11" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr"/>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr"/>
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E48" s="13" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F47" s="14" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="G47" s="13" t="inlineStr"/>
-      <c r="H47" s="12" t="inlineStr">
+      <c r="G48" s="13" t="inlineStr"/>
+      <c r="H48" s="12" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="17" t="inlineStr">
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Lista com os alimentos acrescentados até agora — não é uma lista completa. Use a skill 'adicionar-alimento' (ex.: "adicione sucrilhos") para ir acrescentando novos itens aos poucos. A coluna 'Gostoso' é sua — escolha do menu suspenso; o valor é preservado mesmo quando a planilha é regenerada por um alimento novo.</t>
         </is>
@@ -2262,20 +2295,20 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A41:H41"/>
     <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G5 G6 G7 G8 G9 G10 G12 G13 G14 G15 G17 G18 G19 G20 G21 G23 G24 G25 G26 G27 G28 G30 G31 G32 G33 G34 G35 G37 G38 G39 G41 G42 G43 G44 G45 G47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Escolha uma opção do menu (ou deixe em branco)." type="list" errorStyle="warning">
+    <dataValidation sqref="G5 G6 G7 G8 G9 G10 G12 G13 G14 G15 G16 G18 G19 G20 G21 G22 G24 G25 G26 G27 G28 G29 G31 G32 G33 G34 G35 G36 G38 G39 G40 G42 G43 G44 G45 G46 G48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Escolha uma opção do menu (ou deixe em branco)." type="list" errorStyle="warning">
       <formula1>"Ruim,Normal,Bom,Muito bom"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3964,7 +3997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4442,7 +4475,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Leite desnatado</t>
+          <t>Pão francês integral (multigrãos)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -4516,7 +4549,7 @@
       <c r="J7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Ovo</t>
+          <t>Pão francês integral (multigrãos)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -4526,7 +4559,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Queijo branco frescal</t>
+          <t>Leite desnatado</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -4596,7 +4629,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Leite desnatado</t>
+          <t>Ovo</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -4606,7 +4639,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Queijo frescal light</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -4680,7 +4713,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Queijo branco frescal</t>
+          <t>Leite desnatado</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -4690,7 +4723,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Queijo frescal light</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -4760,7 +4793,7 @@
       <c r="J10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Queijo frescal light</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -4770,7 +4803,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -4830,7 +4863,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Queijo frescal light</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -4840,7 +4873,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -4862,12 +4895,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Peixe</t>
+          <t>Pão francês integral (multigrãos)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Proteínas</t>
+          <t>Grãos e Cereais</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4877,34 +4910,34 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>150 g</t>
+          <t>1 unidade (~67 g)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3x/semana</t>
+          <t>1x/dia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Fonte de ômega-3</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Rótulo real (porção 50 g/meia unidade): 120 kcal, 208 mg de sódio, 1,6 g de fibras, sem açúcar adicionado. Com centeio, gergelim e linhaça — boa fonte de fibra, mas sódio moderado como a maioria dos pães; contém glúten.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -4914,7 +4947,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -4936,7 +4969,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Frango sem pele</t>
+          <t>Peixe</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4956,10 +4989,14 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>quase todo dia</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Fonte de ômega-3</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
@@ -4974,7 +5011,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -4984,7 +5021,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -5006,7 +5043,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carne vermelha magra</t>
+          <t>Frango sem pele</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5016,7 +5053,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5026,14 +5063,10 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1x/semana</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Preferir cortes magros</t>
-        </is>
-      </c>
+          <t>quase todo dia</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
@@ -5048,7 +5081,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -5058,7 +5091,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -5080,7 +5113,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ovo</t>
+          <t>Carne vermelha magra</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5090,25 +5123,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>150 g</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>até 5x/semana</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>1x/semana</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Preferir cortes magros</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>X</t>
@@ -5122,7 +5155,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -5132,7 +5165,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Mussarela</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -5154,7 +5187,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Feijão / leguminosas</t>
+          <t>Ovo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5169,16 +5202,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1 concha</t>
+          <t>1 unidade</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1x/dia</t>
+          <t>até 5x/semana</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>X</t>
@@ -5192,7 +5229,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -5202,7 +5239,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -5224,12 +5261,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leite desnatado</t>
+          <t>Feijão / leguminosas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Laticínios</t>
+          <t>Proteínas</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5239,7 +5276,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 concha</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5248,21 +5285,21 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Mussarela</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -5272,7 +5309,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -5294,7 +5331,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Queijo branco frescal</t>
+          <t>Leite desnatado</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5309,19 +5346,15 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>30 g</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
-        </is>
-      </c>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>X</t>
@@ -5336,12 +5369,12 @@
       <c r="J18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -5358,7 +5391,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Queijo frescal light</t>
+          <t>Queijo branco frescal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5373,7 +5406,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>30 g (1 fatia)</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5383,7 +5416,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Rótulo real: 41 kcal e 105 mg de sódio por porção (bem abaixo de queijos comuns), 1,5 g de gordura saturada, sem açúcar adicionado. Contém lactose; sem glúten; pode conter soja.</t>
+          <t>Tipo fresco (ex.: Minas frescal), sem cura/salga pesada — bem menos sódio e gordura que queijos curados. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5400,12 +5433,12 @@
       <c r="J19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
           <t>Suco natural sem açúcar</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -5422,7 +5455,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mussarela</t>
+          <t>Queijo frescal light</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5432,22 +5465,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>30 g</t>
+          <t>30 g (1 fatia)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2x/semana</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Rótulo real: 41 kcal e 105 mg de sódio por porção (bem abaixo de queijos comuns), 1,5 g de gordura saturada, sem açúcar adicionado. Contém lactose; sem glúten; pode conter soja.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5464,12 +5497,12 @@
       <c r="J20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -5486,7 +5519,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Iogurte natural (desnatado, sem açúcar)</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5496,22 +5529,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1 unidade</t>
+          <t>30 g</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1x/dia</t>
+          <t>2x/semana</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Prefira sempre a versão sem açúcar adicionado</t>
+          <t>Mais gordura saturada e sódio que o queijo branco frescal; prefira o frescal no dia a dia. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5528,12 +5561,12 @@
       <c r="J21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -5550,7 +5583,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Iogurte natural (desnatado, sem açúcar)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5560,22 +5593,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1 colher de sopa (≈15 g)</t>
+          <t>1 unidade</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2x/semana</t>
+          <t>1x/dia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Prefira sempre a versão sem açúcar adicionado</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5592,12 +5625,12 @@
       <c r="J22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -5614,58 +5647,54 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Laticínios</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>1 colher de sopa (≈15 g)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -5682,7 +5711,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5692,25 +5721,25 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>X</t>
@@ -5724,6 +5753,16 @@
       <c r="J24" t="inlineStr">
         <is>
           <t>X</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Manteiga</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -5740,7 +5779,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5750,32 +5789,40 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>Doces e Sobremesas|Jantar</t>
@@ -5790,7 +5837,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5800,24 +5847,20 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>X</t>
@@ -5844,7 +5887,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5854,22 +5897,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5898,7 +5941,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5923,31 +5966,31 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Bebida alcoólica</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Doces e Sobremesas</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5967,24 +6010,16 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>X</t>
@@ -5994,7 +6029,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6017,20 +6052,36 @@
           <t>evitar</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6040,24 +6091,20 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10 g</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
@@ -6070,47 +6117,47 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Azeite de oliva extra virgem</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gorduras e Temperos</t>
+          <t>Doces e Sobremesas</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1-2 colheres de sopa</t>
+          <t>10 g</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6120,37 +6167,37 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6160,41 +6207,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>todos os dias</t>
+          <t>evitar</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Preferir azeite</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6204,22 +6247,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>todos os dias</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+          <t>Somar sal de cozinha + industrializados</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -6238,7 +6281,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6248,20 +6291,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
@@ -6278,50 +6325,90 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Gorduras e Temperos</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>à vontade</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>X</t>
         </is>

</xml_diff>

<commit_message>
Adiciona iogurte grego zero (Vigor) e altura de linha automática
- planilha/dados_alimentos.json: novo item "Iogurte grego zero" (marca
  Vigor, Laticínios, Liberado), com dados reais do rótulo (50 kcal,
  6,8g proteína, sem lactose, zero açúcar/gordura adicionados)
- planilha/gerar_planilha.py: novas funções calc_row_height/estimar_linhas
  que calculam a altura de cada linha a partir do tamanho real do texto
  (em vez de altura fixa), aplicadas nas abas "Cuidados na Alimentação",
  "Plano Geral - Restaurante", "Alimentos e Quantidades" e "Fontes e
  Referências" — corrige rótulos/observações mais longos que antes
  ficavam cortados. A aba "Montar Refeição" mantém altura fixa (colunas
  preenchidas por fórmula, texto real só existe após o Excel calcular)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -719,7 +719,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="46" customHeight="1">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Perfil de risco atual</t>
@@ -731,7 +731,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="46" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Reduzir</t>
@@ -743,7 +743,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Reduzir</t>
@@ -755,7 +755,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Reduzir</t>
@@ -767,7 +767,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Reduzir</t>
@@ -779,7 +779,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Priorizar</t>
@@ -791,7 +791,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Priorizar</t>
@@ -803,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Priorizar</t>
@@ -815,7 +815,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Atenção especial — triglicerídeos</t>
@@ -827,7 +827,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
+    <row r="12" ht="64" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Atenção especial — LDL</t>
@@ -839,7 +839,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="46" customHeight="1">
+    <row r="13" ht="78" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Aviso pendente — função renal</t>
@@ -851,7 +851,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
+    <row r="14" ht="50" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Medicações em uso (receita 03/09/2026)</t>
@@ -863,7 +863,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="46" customHeight="1">
+    <row r="15" ht="64" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Interação medicamentosa — Ticagrelor</t>
@@ -875,7 +875,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="64" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Interação medicamentosa — Enalapril</t>
@@ -887,7 +887,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="46" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Interação medicamentosa — Aspirina + Ticagrelor</t>
@@ -899,7 +899,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="46" customHeight="1">
+    <row r="18" ht="50" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Interação medicamentosa — Rosucor (estatina)</t>
@@ -911,7 +911,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="46" customHeight="1">
+    <row r="19" ht="50" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Reabilitação cardíaca</t>
@@ -923,7 +923,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="46" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Leitura de rótulos</t>
@@ -975,7 +975,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Modelo de prato</t>
@@ -987,7 +987,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>O que pedir</t>
@@ -999,7 +999,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>O que evitar</t>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Perguntas úteis ao garçom</t>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Exemplos de pratos que funcionam</t>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Em festas/eventos</t>
@@ -1061,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1296,7 +1296,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="64" customHeight="1">
       <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Toranja / grapefruit</t>
@@ -1447,7 +1447,7 @@
       <c r="G15" s="13" t="inlineStr"/>
       <c r="H15" s="12" t="inlineStr"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="64" customHeight="1">
       <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Pão francês integral (multigrãos)</t>
@@ -1666,7 +1666,7 @@
       <c r="G24" s="13" t="inlineStr"/>
       <c r="H24" s="12" t="inlineStr"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="50" customHeight="1">
       <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Queijo branco frescal</t>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="50" customHeight="1">
       <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Queijo frescal light</t>
@@ -1728,7 +1728,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="50" customHeight="1">
       <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Mussarela</t>
@@ -1786,190 +1786,194 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="50" customHeight="1">
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Requeijão</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr"/>
+          <t>Iogurte grego zero</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Vigor</t>
+        </is>
+      </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>1 colher de sopa (≈15 g)</t>
+          <t>90 g (1 pote)</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F29" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G29" s="13" t="inlineStr"/>
       <c r="H29" s="12" t="inlineStr">
         <is>
+          <t>Rótulo real: 50 kcal, 6,8 g de proteína (bem mais que iogurte comum), 0,2 g de gordura, 51 mg de sódio, zero adição de açúcar/gordura, sem lactose. Contém edulcorantes (sucralose e ciclamato).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr"/>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>1 colher de sopa (≈15 g)</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr"/>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
           <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Bebidas</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="11" t="n"/>
-      <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
-      <c r="H30" s="11" t="n"/>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr"/>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>à vontade</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr"/>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F32" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+      <c r="H32" s="12" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr"/>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G33" s="13" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr"/>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr"/>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F34" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr"/>
-      <c r="H34" s="12" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+      <c r="H34" s="12" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr"/>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>3x/semana</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G35" s="13" t="inlineStr"/>
       <c r="H35" s="12" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="64" customHeight="1">
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr"/>
@@ -1991,57 +1995,57 @@
       <c r="G36" s="13" t="inlineStr"/>
       <c r="H36" s="12" t="inlineStr">
         <is>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Bebida alcoólica</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr"/>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr"/>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
           <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>Doces e Sobremesas</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="11" t="n"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>Açúcar refinado</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr"/>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr"/>
-      <c r="H38" s="12" t="inlineStr">
-        <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="11" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr"/>
@@ -2061,233 +2065,262 @@
         </is>
       </c>
       <c r="G39" s="13" t="inlineStr"/>
-      <c r="H39" s="12" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr"/>
       <c r="D40" s="13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr"/>
+      <c r="H40" s="12" t="inlineStr"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Chocolate amargo (70%+)</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr"/>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
           <t>10 g</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E41" s="13" t="inlineStr">
         <is>
           <t>2x/semana</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>Moderar</t>
         </is>
       </c>
-      <c r="G40" s="13" t="inlineStr"/>
-      <c r="H40" s="12" t="inlineStr">
+      <c r="G41" s="13" t="inlineStr"/>
+      <c r="H41" s="12" t="inlineStr">
         <is>
           <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Gorduras e Temperos</t>
         </is>
       </c>
-      <c r="B41" s="11" t="n"/>
-      <c r="C41" s="11" t="n"/>
-      <c r="D41" s="11" t="n"/>
-      <c r="E41" s="11" t="n"/>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
-      <c r="H41" s="11" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>Azeite de oliva extra virgem</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr"/>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>1-2 colheres de sopa</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F42" s="14" t="inlineStr">
-        <is>
-          <t>Liberado</t>
-        </is>
-      </c>
-      <c r="G42" s="13" t="inlineStr"/>
-      <c r="H42" s="12" t="inlineStr"/>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr"/>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F43" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="G43" s="13" t="inlineStr"/>
-      <c r="H43" s="12" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
+      <c r="H43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr"/>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F44" s="15" t="inlineStr">
-        <is>
-          <t>Moderar</t>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="G44" s="13" t="inlineStr"/>
       <c r="H44" s="12" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
+          <t>Preferir azeite</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr"/>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F45" s="16" t="inlineStr">
-        <is>
-          <t>Evitar</t>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr"/>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
+          <t>Somar sal de cozinha + industrializados</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr"/>
       <c r="D46" s="13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="inlineStr"/>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr"/>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E47" s="13" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F46" s="14" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="G46" s="13" t="inlineStr"/>
-      <c r="H46" s="12" t="inlineStr"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="G47" s="13" t="inlineStr"/>
+      <c r="H47" s="12" t="inlineStr"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="B47" s="11" t="n"/>
-      <c r="C47" s="11" t="n"/>
-      <c r="D47" s="11" t="n"/>
-      <c r="E47" s="11" t="n"/>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
-      <c r="H47" s="11" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="11" t="n"/>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr"/>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr"/>
+      <c r="D49" s="13" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E49" s="13" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F48" s="14" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="G48" s="13" t="inlineStr"/>
-      <c r="H48" s="12" t="inlineStr">
+      <c r="G49" s="13" t="inlineStr"/>
+      <c r="H49" s="12" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="40" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Lista com os alimentos acrescentados até agora — não é uma lista completa. Use a skill 'adicionar-alimento' (ex.: "adicione sucrilhos") para ir acrescentando novos itens aos poucos. A coluna 'Gostoso' é sua — escolha do menu suspenso; o valor é preservado mesmo quando a planilha é regenerada por um alimento novo.</t>
         </is>
@@ -2295,20 +2328,20 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G5 G6 G7 G8 G9 G10 G12 G13 G14 G15 G16 G18 G19 G20 G21 G22 G24 G25 G26 G27 G28 G29 G31 G32 G33 G34 G35 G36 G38 G39 G40 G42 G43 G44 G45 G46 G48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Escolha uma opção do menu (ou deixe em branco)." type="list" errorStyle="warning">
+    <dataValidation sqref="G5 G6 G7 G8 G9 G10 G12 G13 G14 G15 G16 G18 G19 G20 G21 G22 G24 G25 G26 G27 G28 G29 G30 G32 G33 G34 G35 G36 G37 G39 G40 G41 G43 G44 G45 G46 G47 G49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Escolha uma opção do menu (ou deixe em branco)." type="list" errorStyle="warning">
       <formula1>"Ruim,Normal,Bom,Muito bom"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3290,7 +3323,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="32" t="n">
         <v>1</v>
       </c>
@@ -3320,7 +3353,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="32" t="n">
         <v>2</v>
       </c>
@@ -3350,7 +3383,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="32" t="n">
         <v>3</v>
       </c>
@@ -3380,7 +3413,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="44" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="32" t="n">
         <v>4</v>
       </c>
@@ -3410,7 +3443,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="32" t="n">
         <v>5</v>
       </c>
@@ -3440,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="32" t="n">
         <v>6</v>
       </c>
@@ -3470,7 +3503,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="44" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="32" t="n">
         <v>7</v>
       </c>
@@ -3500,7 +3533,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1">
+    <row r="11" ht="50" customHeight="1">
       <c r="A11" s="32" t="n">
         <v>8</v>
       </c>
@@ -3530,7 +3563,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="44" customHeight="1">
+    <row r="12" ht="50" customHeight="1">
       <c r="A12" s="32" t="n">
         <v>9</v>
       </c>
@@ -3560,7 +3593,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="32" t="n">
         <v>10</v>
       </c>
@@ -3590,7 +3623,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="32" t="n">
         <v>11</v>
       </c>
@@ -3620,7 +3653,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="32" t="n">
         <v>12</v>
       </c>
@@ -3650,7 +3683,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="32" t="n">
         <v>13</v>
       </c>
@@ -3680,7 +3713,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="32" t="n">
         <v>14</v>
       </c>
@@ -3710,7 +3743,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="44" customHeight="1">
+    <row r="18" ht="50" customHeight="1">
       <c r="A18" s="32" t="n">
         <v>15</v>
       </c>
@@ -3740,7 +3773,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="44" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="32" t="n">
         <v>16</v>
       </c>
@@ -3770,7 +3803,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="32" t="n">
         <v>17</v>
       </c>
@@ -3800,7 +3833,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="44" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="32" t="n">
         <v>18</v>
       </c>
@@ -3830,7 +3863,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="44" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="32" t="n">
         <v>19</v>
       </c>
@@ -3860,7 +3893,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="44" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="32" t="n">
         <v>20</v>
       </c>
@@ -3890,7 +3923,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="44" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="32" t="n">
         <v>21</v>
       </c>
@@ -3920,7 +3953,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="44" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="32" t="n">
         <v>22</v>
       </c>
@@ -3997,7 +4030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4873,7 +4906,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte grego zero</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -4947,7 +4980,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -5011,7 +5044,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Iogurte grego zero</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -5021,7 +5054,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -5081,7 +5114,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -5091,7 +5124,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -5155,7 +5188,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Vegetais e verduras em geral</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -5165,7 +5198,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -5229,7 +5262,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Uva</t>
+          <t>Vegetais e verduras em geral</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -5239,7 +5272,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Mussarela</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -5299,7 +5332,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Manga</t>
+          <t>Uva</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -5309,7 +5342,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -5369,12 +5402,12 @@
       <c r="J18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Mussarela</t>
+          <t>Manga</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -5433,12 +5466,12 @@
       <c r="J19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Mussarela</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -5497,12 +5530,12 @@
       <c r="J20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
+          <t>Requeijão</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
           <t>Suco natural sem açúcar</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -5561,12 +5594,12 @@
       <c r="J21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Toranja / grapefruit</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -5625,12 +5658,12 @@
       <c r="J22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -5647,7 +5680,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Requeijão</t>
+          <t>Iogurte grego zero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5657,22 +5690,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1 colher de sopa (≈15 g)</t>
+          <t>90 g (1 pote)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2x/semana</t>
+          <t>1x/dia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+          <t>Rótulo real: 50 kcal, 6,8 g de proteína (bem mais que iogurte comum), 0,2 g de gordura, 51 mg de sódio, zero adição de açúcar/gordura, sem lactose. Contém edulcorantes (sucralose e ciclamato).</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5689,12 +5722,12 @@
       <c r="J23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -5711,58 +5744,54 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Requeijão</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bebidas</t>
+          <t>Laticínios</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>1 colher de sopa (≈15 g)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Rico em gordura saturada e sódio; prefira a versão light. Sugestão gerada por IA — confirmar com nutricionista/cardiologista.</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -5779,7 +5808,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Refrigerante zero</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5789,25 +5818,25 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>à vontade</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>X</t>
@@ -5821,6 +5850,16 @@
       <c r="J25" t="inlineStr">
         <is>
           <t>X</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Manteiga</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -5837,7 +5876,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Café sem açúcar</t>
+          <t>Refrigerante zero</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5847,32 +5886,40 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1 xícara</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2x/dia</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t>Gorduras e Temperos|Jantar</t>
@@ -5887,7 +5934,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Suco natural sem açúcar</t>
+          <t>Café sem açúcar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5897,24 +5944,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>1 xícara</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3x/semana</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Preferir a fruta inteira, que tem mais fibra</t>
-        </is>
-      </c>
+          <t>2x/dia</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>X</t>
@@ -5941,7 +5984,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Suco de toranja / grapefruit</t>
+          <t>Suco natural sem açúcar</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5951,22 +5994,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>3x/semana</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+          <t>Preferir a fruta inteira, que tem mais fibra</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5985,7 +6028,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bebida alcoólica</t>
+          <t>Suco de toranja / grapefruit</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6010,31 +6053,31 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Interage com o Ticagrelor (estudo mostrou quase o dobro do nível do remédio no sangue); a bula diz que não é esperado ser clinicamente relevante p/ a maioria, mas orienta evitar — mais seguro evitar, já que você toma 2 antiagregantes. Ver aba Fontes e Referências.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Açúcar refinado</t>
+          <t>Bebida alcoólica</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Doces e Sobremesas</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6054,24 +6097,16 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Impacto direto nos triglicerídeos</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Piora diretamente os triglicerídeos; soma-se ao risco de sangramento da Aspirina + Ticagrelor.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>X</t>
@@ -6081,7 +6116,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Doces industrializados</t>
+          <t>Açúcar refinado</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6104,20 +6139,36 @@
           <t>evitar</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Impacto direto nos triglicerídeos</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Chocolate amargo (70%+)</t>
+          <t>Doces industrializados</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6127,24 +6178,20 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10 g</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2x/semana</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
-        </is>
-      </c>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
@@ -6157,47 +6204,47 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Azeite de oliva extra virgem</t>
+          <t>Chocolate amargo (70%+)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gorduras e Temperos</t>
+          <t>Doces e Sobremesas</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1-2 colheres de sopa</t>
+          <t>10 g</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1x/dia</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>2x/semana</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Sugestão gerada por IA — confirmar com nutricionista/cardiologista</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Manteiga</t>
+          <t>Azeite de oliva extra virgem</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6207,37 +6254,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Liberado</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1-2 colheres de sopa</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>evitar</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Preferir azeite</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>1x/dia</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sal</t>
+          <t>Manteiga</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6247,41 +6294,37 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Moderar</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>&lt; 5 g no total</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>todos os dias</t>
+          <t>evitar</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Somar sal de cozinha + industrializados</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Preferir azeite</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sal light / substituto de sal (cloreto de potássio)</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6291,22 +6334,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Evitar</t>
+          <t>Moderar</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>&lt; 5 g no total</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>evitar</t>
+          <t>todos os dias</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+          <t>Somar sal de cozinha + industrializados</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -6325,7 +6368,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ervas e temperos naturais</t>
+          <t>Sal light / substituto de sal (cloreto de potássio)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6335,20 +6378,24 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Liberado</t>
+          <t>Evitar</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>à vontade</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>todos os dias</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>evitar</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Enalapril já tende a elevar o potássio; combinado com esse produto o risco de hipercalemia aumenta, ainda mais com a função renal pendente.</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
@@ -6365,50 +6412,90 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>Ervas e temperos naturais</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Gorduras e Temperos</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Liberado</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>à vontade</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>todos os dias</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Vegetais e verduras em geral</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Vegetais e Verduras</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Liberado</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>à vontade</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>todos os dias</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Se entrar anticoagulante na medicação, revisar consumo de verde-escuros ricos em vitamina K</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>X</t>
         </is>

</xml_diff>

<commit_message>
Atualiza aveia com marca Quaker e dados reais do rótulo
- 'Aveia' -> 'Aveia integral em flocos' (marca Quaker), mesma comida já
  cadastrada, agora com dados reais: 110 kcal, 2,8g de fibra (1,2g de
  beta-glucana), sem açúcar adicionado, 0mg de sódio por porção

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B3UbsXJe742GjvUpiD7rC7
</commit_message>
<xml_diff>
--- a/planilha/plano-alimentar-pos-infarto.xlsx
+++ b/planilha/plano-alimentar-pos-infarto.xlsx
@@ -1393,16 +1393,20 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="50" customHeight="1">
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Aveia</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr"/>
+          <t>Aveia integral em flocos</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Quaker</t>
+        </is>
+      </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>2 colheres de sopa</t>
+          <t>2 colheres de sopa (~30 g)</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -1418,7 +1422,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>Ajuda a reduzir colesterol</t>
+          <t>Rótulo real: 110 kcal, 2,8 g de fibra (1,2 g de beta-glucana — a fibra solúvel que ajuda a reduzir o colesterol), sem açúcar adicionado, 0 mg de sódio.</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4275,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Aveia</t>
+          <t>Aveia integral em flocos</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -4414,7 +4418,7 @@
       <c r="J5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Aveia</t>
+          <t>Aveia integral em flocos</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -4788,7 +4792,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aveia</t>
+          <t>Aveia integral em flocos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4803,7 +4807,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2 colheres de sopa</t>
+          <t>2 colheres de sopa (~30 g)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4813,7 +4817,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ajuda a reduzir colesterol</t>
+          <t>Rótulo real: 110 kcal, 2,8 g de fibra (1,2 g de beta-glucana — a fibra solúvel que ajuda a reduzir o colesterol), sem açúcar adicionado, 0 mg de sódio.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>